<commit_message>
Anpassungen und Fixes Temperaturspeicher
</commit_message>
<xml_diff>
--- a/Outputs/konstanterTemperaturspeicher/Fehleranalyse_pypsa_trynsis.xlsx
+++ b/Outputs/konstanterTemperaturspeicher/Fehleranalyse_pypsa_trynsis.xlsx
@@ -477,25 +477,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4.370311356235323</v>
+        <v>4.01778996933056</v>
       </c>
       <c r="C2" t="n">
-        <v>6.606383127538405</v>
+        <v>6.276090975609679</v>
       </c>
       <c r="D2" t="n">
-        <v>15.18735796010126</v>
+        <v>14.31206595526532</v>
       </c>
       <c r="E2" t="n">
-        <v>4.369755511287638</v>
+        <v>4.017234124382876</v>
       </c>
       <c r="F2" t="n">
-        <v>10.04559376391766</v>
+        <v>9.160944283527538</v>
       </c>
       <c r="G2" t="n">
-        <v>0.455286414694339</v>
+        <v>0.4828143209988451</v>
       </c>
       <c r="H2" t="n">
-        <v>20.02945347139875</v>
+        <v>20.02946347139876</v>
       </c>
       <c r="I2" t="n">
         <v>480</v>

</xml_diff>